<commit_message>
Daily attendance processing - 2026-05-13 06:59:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_Urogenital_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_Urogenital_session_analysis.xlsx
@@ -1022,7 +1022,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>39.8%</t>
+          <t>40.1%</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>35.5%</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>108/227</t>
+          <t>163/227</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">

</xml_diff>